<commit_message>
fix: update Appium_Mobile_E2E_Analysis_Report.xlsx generator with descriptive test names
</commit_message>
<xml_diff>
--- a/appium-tests/reports/MediFind_Mobile_E2E_Report.xlsx
+++ b/appium-tests/reports/MediFind_Mobile_E2E_Report.xlsx
@@ -17,7 +17,7 @@
     <t>📱 MediFind Android Mobile E2E Test Execution Summary</t>
   </si>
   <si>
-    <t>Generated On: 24/8/2026, 3:44:33 pm | Environment: Android Emulator / UiAutomator2</t>
+    <t>Generated On: 25/8/2026, 10:03:13 am | Environment: Android Emulator / UiAutomator2</t>
   </si>
   <si>
     <t>Total Test Cases Executed</t>
@@ -811,7 +811,7 @@
         <v>22</v>
       </c>
       <c r="F2" s="8">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>23</v>

</xml_diff>